<commit_message>
02-feature-engineering, minh chung excel
</commit_message>
<xml_diff>
--- a/Chalenge2/reports/eda_summary.xlsx
+++ b/Chalenge2/reports/eda_summary.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\ml_personalNGroup\Group\chalenge2\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48C21974-4D6F-4E60-B587-B69980D67146}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBCA2EF7-A636-4171-B4FD-9014478EE4C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="EDA Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -150,27 +149,12 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -179,14 +163,14 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -614,12 +598,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B92"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="33.1796875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
     </row>
@@ -712,8 +699,8 @@
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A40" s="2"/>
-      <c r="B40" s="3"/>
+      <c r="A40" s="1"/>
+      <c r="B40" s="2"/>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
@@ -863,13 +850,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>